<commit_message>
feat: nouveau rôle AdminEcole - gestion des utilisateurs par école
- Roles.AdminEcole : peut gérer les utilisateurs de ses écoles assignées
- UtilisateurController : accessible à Admin et AdminEcole
  - Index : AdminEcole voit seulement les utilisateurs de ses écoles
  - Create/Edit : AdminEcole ne peut créer/modifier que des Utilisateurs dans ses écoles
  - AdminEcole ne peut pas créer/promouvoir Admin ou AdminEcole
  - Edit : préserve les accès hors-scope de l'AdminEcole lors de la modification
  - Supprimer : AdminEcole ne peut pas supprimer Admin/AdminEcole
- RolesDisponibles : liste dynamique selon le rôle du gestionnaire
- Vues Create/Edit : sélecteur de rôle depuis RolesDisponibles
- AdminEcole cache aussi la section écoles (accès implicite à toutes ses écoles)
- _Layout : menu Utilisateurs visible pour AdminEcole
- Badge distinct : Admin global (rouge), Admin école (jaune), Utilisateur (gris)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Data/ecoles.xlsx
+++ b/Data/ecoles.xlsx
@@ -40,13 +40,25 @@
     <x:t>Les Aigles</x:t>
   </x:si>
   <x:si>
+    <x:t>/uploads/logos/837f56a2-8c28-462c-94d6-929dc124d12f.png</x:t>
+  </x:si>
+  <x:si>
+    <x:t>#1a3a5c</x:t>
+  </x:si>
+  <x:si>
+    <x:t>#d58d10</x:t>
+  </x:si>
+  <x:si>
+    <x:t>École Armand-Corbail</x:t>
+  </x:si>
+  <x:si>
     <x:t/>
   </x:si>
   <x:si>
-    <x:t>#1a3a5c</x:t>
-  </x:si>
-  <x:si>
-    <x:t>#d58d10</x:t>
+    <x:t>#e8a020</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Les Scorpions</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -440,6 +452,26 @@
         <x:v>10</x:v>
       </x:c>
     </x:row>
+    <x:row r="3" spans="1:6">
+      <x:c r="A3" s="0">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="B3" s="0" t="s">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="D3" s="0" t="s">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
+        <x:v>13</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>

<commit_message>
Correctif avant carte entrain
</commit_message>
<xml_diff>
--- a/Data/ecoles.xlsx
+++ b/Data/ecoles.xlsx
@@ -43,10 +43,10 @@
     <x:t>/uploads/logos/837f56a2-8c28-462c-94d6-929dc124d12f.png</x:t>
   </x:si>
   <x:si>
-    <x:t>#1a3a5c</x:t>
-  </x:si>
-  <x:si>
-    <x:t>#c9a646</x:t>
+    <x:t>#1c2f5c</x:t>
+  </x:si>
+  <x:si>
+    <x:t>#e0be4a</x:t>
   </x:si>
   <x:si>
     <x:t>[{"Type":"Facebook","Url":"https://www.facebook.com/profile.php?id=100057229281252","Label":null},{"Type":"Instagram","Url":"https://www.instagram.com/aigles.rseq.amitie/","Label":null}]</x:t>
@@ -61,10 +61,10 @@
     <x:t>/uploads/logos/ccde6cd6-7342-4fd0-9274-890a0db77e5e.avif</x:t>
   </x:si>
   <x:si>
-    <x:t>#ffda24</x:t>
-  </x:si>
-  <x:si>
-    <x:t>#121212</x:t>
+    <x:t>#1f3a6d</x:t>
+  </x:si>
+  <x:si>
+    <x:t>#e3b23c</x:t>
   </x:si>
   <x:si>
     <x:t/>
@@ -478,10 +478,10 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
+        <x:v>15</x:v>
+      </x:c>
+      <x:c r="F3" s="0" t="s">
         <x:v>16</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>15</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
         <x:v>17</x:v>

</xml_diff>

<commit_message>
Page joueur corrigé plus model
</commit_message>
<xml_diff>
--- a/Data/ecoles.xlsx
+++ b/Data/ecoles.xlsx
@@ -50,24 +50,6 @@
   </x:si>
   <x:si>
     <x:t>[{"Type":"Facebook","Url":"https://www.facebook.com/profile.php?id=100057229281252","Label":null},{"Type":"Instagram","Url":"https://www.instagram.com/aigles.rseq.amitie/","Label":null}]</x:t>
-  </x:si>
-  <x:si>
-    <x:t>École Armand-Corbeil</x:t>
-  </x:si>
-  <x:si>
-    <x:t>Les Scorpions</x:t>
-  </x:si>
-  <x:si>
-    <x:t>/uploads/logos/ccde6cd6-7342-4fd0-9274-890a0db77e5e.avif</x:t>
-  </x:si>
-  <x:si>
-    <x:t>#1f3a6d</x:t>
-  </x:si>
-  <x:si>
-    <x:t>#e3b23c</x:t>
-  </x:si>
-  <x:si>
-    <x:t/>
   </x:si>
 </x:sst>
 </file>
@@ -464,29 +446,6 @@
         <x:v>11</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" spans="1:7">
-      <x:c r="A3" s="0">
-        <x:v>2</x:v>
-      </x:c>
-      <x:c r="B3" s="0" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>13</x:v>
-      </x:c>
-      <x:c r="D3" s="0" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>15</x:v>
-      </x:c>
-      <x:c r="F3" s="0" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
   <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>

</xml_diff>